<commit_message>
integrated regrid in place of attom for property data
</commit_message>
<xml_diff>
--- a/agent-1/inputs/agent1_search_request.xlsx
+++ b/agent-1/inputs/agent1_search_request.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ananya.Mehta\OneDrive - Parkar\Desktop\redpine-ai\agent-1\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2975D7FB-B232-4069-B0D2-A8DC8F7EC3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{917DF480-C375-468E-9475-79B6EB3D7A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
     <t>Year Built Range</t>
   </si>
   <si>
-    <t>Orlando, Florida</t>
+    <t>Dallas, Texas</t>
   </si>
 </sst>
 </file>

</xml_diff>